<commit_message>
Update appendices, forecasts, figures and scripts
Bulk refresh of outcome appendices, forecasts, figures and analysis scripts. Updated numerous Forecasts_with_best_model and Forecasts_with_intervals CSVs, supplementary appendix images and tables, and publish/figure data; edited External_pertussis_decision_support.md (best-model selections, summary stats and source paths). Replaced/added Appendix assets (including flow_diagram.png and external pertussis PNG), updated Data/Population/province.xlsx, refreshed ScriptAnalysis R scripts and temporary RData files, and removed an outdated PDF and Rhistory. This commit brings documentation, outputs and scripts into sync with the latest analysis results.
</commit_message>
<xml_diff>
--- a/Outcome/Appendix/Tables/Best_model_outcome.xlsx
+++ b/Outcome/Appendix/Tables/Best_model_outcome.xlsx
@@ -485,7 +485,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>7.01</v>
+        <v>5.7</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -502,7 +502,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>-2.91</v>
+        <v>2.42</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -519,7 +519,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>6.66</v>
+        <v>5.29</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -536,7 +536,7 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>1.22</v>
+        <v>0.36</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -553,7 +553,7 @@
         <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>-12.84</v>
+        <v>-12.97</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -570,7 +570,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>-3.66</v>
+        <v>-4.28</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -587,7 +587,7 @@
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>4.53</v>
+        <v>3.48</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -604,7 +604,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="n">
-        <v>4.8</v>
+        <v>4.83</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -621,7 +621,7 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>0.44</v>
+        <v>-0.36</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -638,7 +638,7 @@
         <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>0.08</v>
+        <v>0.13</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -655,7 +655,7 @@
         <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>2.92</v>
+        <v>3.28</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -672,7 +672,7 @@
         <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>-6.59</v>
+        <v>-6.36</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -689,7 +689,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>0.49</v>
+        <v>0.54</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -706,7 +706,7 @@
         <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>-2.16</v>
+        <v>-2.06</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -723,7 +723,7 @@
         <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>2.33</v>
+        <v>2.16</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -740,7 +740,7 @@
         <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>-4.58</v>
+        <v>-4.22</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -757,7 +757,7 @@
         <v>9</v>
       </c>
       <c r="C18" t="n">
-        <v>2.44</v>
+        <v>2.39</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -774,7 +774,7 @@
         <v>10</v>
       </c>
       <c r="C19" t="n">
-        <v>3.41</v>
+        <v>3.4</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -791,7 +791,7 @@
         <v>11</v>
       </c>
       <c r="C20" t="n">
-        <v>-3.75</v>
+        <v>-3.8</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
         <v>12</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.41</v>
+        <v>-0.39</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -825,7 +825,7 @@
         <v>13</v>
       </c>
       <c r="C22" t="n">
-        <v>0.56</v>
+        <v>0.47</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -842,7 +842,7 @@
         <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>1.14</v>
+        <v>-0.03</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -859,7 +859,7 @@
         <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>6.53</v>
+        <v>11.71</v>
       </c>
       <c r="D24" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         <v>9</v>
       </c>
       <c r="C25" t="n">
-        <v>-4.97</v>
+        <v>-5.4</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -893,7 +893,7 @@
         <v>10</v>
       </c>
       <c r="C26" t="n">
-        <v>-1.07</v>
+        <v>-2.01</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -910,7 +910,7 @@
         <v>11</v>
       </c>
       <c r="C27" t="n">
-        <v>0.36</v>
+        <v>-0.55</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -927,7 +927,7 @@
         <v>12</v>
       </c>
       <c r="C28" t="n">
-        <v>-2.66</v>
+        <v>-3.05</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -944,7 +944,7 @@
         <v>13</v>
       </c>
       <c r="C29" t="n">
-        <v>0.67</v>
+        <v>-0.67</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -961,7 +961,7 @@
         <v>6</v>
       </c>
       <c r="C30" t="n">
-        <v>0.94</v>
+        <v>0.72</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -978,7 +978,7 @@
         <v>8</v>
       </c>
       <c r="C31" t="n">
-        <v>2.84</v>
+        <v>3.01</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
         <v>9</v>
       </c>
       <c r="C32" t="n">
-        <v>6.09</v>
+        <v>5.71</v>
       </c>
       <c r="D32" t="n">
         <v>1</v>
@@ -1012,7 +1012,7 @@
         <v>10</v>
       </c>
       <c r="C33" t="n">
-        <v>3.73</v>
+        <v>3.98</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1029,7 +1029,7 @@
         <v>11</v>
       </c>
       <c r="C34" t="n">
-        <v>-11.8</v>
+        <v>-11.59</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -1046,7 +1046,7 @@
         <v>12</v>
       </c>
       <c r="C35" t="n">
-        <v>2.86</v>
+        <v>2.81</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1063,7 +1063,7 @@
         <v>13</v>
       </c>
       <c r="C36" t="n">
-        <v>-4.65</v>
+        <v>-4.64</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1080,7 +1080,7 @@
         <v>6</v>
       </c>
       <c r="C37" t="n">
-        <v>0.77</v>
+        <v>-0.94</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1097,10 +1097,10 @@
         <v>8</v>
       </c>
       <c r="C38" t="n">
-        <v>1.39</v>
+        <v>9.52</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" t="s">
         <v>7</v>
@@ -1114,7 +1114,7 @@
         <v>9</v>
       </c>
       <c r="C39" t="n">
-        <v>-1.15</v>
+        <v>-3.55</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -1131,7 +1131,7 @@
         <v>10</v>
       </c>
       <c r="C40" t="n">
-        <v>2.34</v>
+        <v>1.21</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1148,7 +1148,7 @@
         <v>11</v>
       </c>
       <c r="C41" t="n">
-        <v>-9.38</v>
+        <v>-10.94</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -1165,10 +1165,10 @@
         <v>12</v>
       </c>
       <c r="C42" t="n">
-        <v>7.27</v>
+        <v>7.56</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E42" t="s">
         <v>7</v>
@@ -1182,7 +1182,7 @@
         <v>13</v>
       </c>
       <c r="C43" t="n">
-        <v>-1.24</v>
+        <v>-2.86</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
@@ -1199,7 +1199,7 @@
         <v>6</v>
       </c>
       <c r="C44" t="n">
-        <v>1.69</v>
+        <v>1.13</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
@@ -1216,7 +1216,7 @@
         <v>8</v>
       </c>
       <c r="C45" t="n">
-        <v>-7.73</v>
+        <v>-6.4</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -1233,7 +1233,7 @@
         <v>9</v>
       </c>
       <c r="C46" t="n">
-        <v>5.33</v>
+        <v>5.08</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
@@ -1267,7 +1267,7 @@
         <v>11</v>
       </c>
       <c r="C48" t="n">
-        <v>-0.49</v>
+        <v>-0.38</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
@@ -1284,7 +1284,7 @@
         <v>12</v>
       </c>
       <c r="C49" t="n">
-        <v>-7.49</v>
+        <v>-8.24</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -1301,7 +1301,7 @@
         <v>13</v>
       </c>
       <c r="C50" t="n">
-        <v>5.5</v>
+        <v>5.62</v>
       </c>
       <c r="D50" t="n">
         <v>1</v>
@@ -1318,7 +1318,7 @@
         <v>6</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.59</v>
+        <v>-0.07</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -1335,7 +1335,7 @@
         <v>8</v>
       </c>
       <c r="C52" t="n">
-        <v>-4.72</v>
+        <v>-4.36</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
@@ -1352,7 +1352,7 @@
         <v>9</v>
       </c>
       <c r="C53" t="n">
-        <v>-4.41</v>
+        <v>-4.75</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -1369,7 +1369,7 @@
         <v>10</v>
       </c>
       <c r="C54" t="n">
-        <v>7.24</v>
+        <v>6.9</v>
       </c>
       <c r="D54" t="n">
         <v>1</v>
@@ -1386,7 +1386,7 @@
         <v>11</v>
       </c>
       <c r="C55" t="n">
-        <v>4.52</v>
+        <v>4.22</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -1403,7 +1403,7 @@
         <v>12</v>
       </c>
       <c r="C56" t="n">
-        <v>-4.29</v>
+        <v>-4.15</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -1420,7 +1420,7 @@
         <v>13</v>
       </c>
       <c r="C57" t="n">
-        <v>2.25</v>
+        <v>2.22</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -1437,7 +1437,7 @@
         <v>6</v>
       </c>
       <c r="C58" t="n">
-        <v>3.33</v>
+        <v>4.16</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -1454,7 +1454,7 @@
         <v>8</v>
       </c>
       <c r="C59" t="n">
-        <v>-1.62</v>
+        <v>-6.69</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -1471,7 +1471,7 @@
         <v>9</v>
       </c>
       <c r="C60" t="n">
-        <v>-4.96</v>
+        <v>-2.92</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -1488,7 +1488,7 @@
         <v>10</v>
       </c>
       <c r="C61" t="n">
-        <v>3.71</v>
+        <v>4.47</v>
       </c>
       <c r="D61" t="n">
         <v>1</v>
@@ -1505,7 +1505,7 @@
         <v>11</v>
       </c>
       <c r="C62" t="n">
-        <v>-3.49</v>
+        <v>-3.24</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -1522,7 +1522,7 @@
         <v>12</v>
       </c>
       <c r="C63" t="n">
-        <v>0.3</v>
+        <v>0.47</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -1539,7 +1539,7 @@
         <v>13</v>
       </c>
       <c r="C64" t="n">
-        <v>2.73</v>
+        <v>3.75</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -1556,7 +1556,7 @@
         <v>6</v>
       </c>
       <c r="C65" t="n">
-        <v>-0.92</v>
+        <v>0.23</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -1573,7 +1573,7 @@
         <v>8</v>
       </c>
       <c r="C66" t="n">
-        <v>6.24</v>
+        <v>5.49</v>
       </c>
       <c r="D66" t="n">
         <v>1</v>
@@ -1590,7 +1590,7 @@
         <v>9</v>
       </c>
       <c r="C67" t="n">
-        <v>-6.33</v>
+        <v>-6.51</v>
       </c>
       <c r="D67" t="n">
         <v>0</v>
@@ -1607,7 +1607,7 @@
         <v>10</v>
       </c>
       <c r="C68" t="n">
-        <v>0.11</v>
+        <v>-0.11</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
         <v>11</v>
       </c>
       <c r="C69" t="n">
-        <v>0.31</v>
+        <v>0.01</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -1641,7 +1641,7 @@
         <v>12</v>
       </c>
       <c r="C70" t="n">
-        <v>2.12</v>
+        <v>2.15</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
@@ -1658,7 +1658,7 @@
         <v>13</v>
       </c>
       <c r="C71" t="n">
-        <v>-1.54</v>
+        <v>-1.26</v>
       </c>
       <c r="D71" t="n">
         <v>0</v>
@@ -1675,7 +1675,7 @@
         <v>6</v>
       </c>
       <c r="C72" t="n">
-        <v>1.02</v>
+        <v>1.88</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
@@ -1692,10 +1692,10 @@
         <v>8</v>
       </c>
       <c r="C73" t="n">
-        <v>6.45</v>
+        <v>1.09</v>
       </c>
       <c r="D73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E73" t="s">
         <v>21</v>
@@ -1709,7 +1709,7 @@
         <v>9</v>
       </c>
       <c r="C74" t="n">
-        <v>-2.38</v>
+        <v>-1.76</v>
       </c>
       <c r="D74" t="n">
         <v>0</v>
@@ -1726,7 +1726,7 @@
         <v>10</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.2</v>
+        <v>0.81</v>
       </c>
       <c r="D75" t="n">
         <v>0</v>
@@ -1743,7 +1743,7 @@
         <v>11</v>
       </c>
       <c r="C76" t="n">
-        <v>-11.1</v>
+        <v>-10.47</v>
       </c>
       <c r="D76" t="n">
         <v>0</v>
@@ -1760,7 +1760,7 @@
         <v>12</v>
       </c>
       <c r="C77" t="n">
-        <v>1.61</v>
+        <v>2.97</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
@@ -1777,10 +1777,10 @@
         <v>13</v>
       </c>
       <c r="C78" t="n">
-        <v>4.61</v>
+        <v>5.47</v>
       </c>
       <c r="D78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E78" t="s">
         <v>21</v>
@@ -1794,7 +1794,7 @@
         <v>6</v>
       </c>
       <c r="C79" t="n">
-        <v>3.34</v>
+        <v>-0.73</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
@@ -1811,7 +1811,7 @@
         <v>8</v>
       </c>
       <c r="C80" t="n">
-        <v>-14.29</v>
+        <v>-7.8</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
@@ -1828,7 +1828,7 @@
         <v>9</v>
       </c>
       <c r="C81" t="n">
-        <v>-1.21</v>
+        <v>-1.94</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -1845,7 +1845,7 @@
         <v>10</v>
       </c>
       <c r="C82" t="n">
-        <v>6.59</v>
+        <v>7.9</v>
       </c>
       <c r="D82" t="n">
         <v>1</v>
@@ -1862,7 +1862,7 @@
         <v>11</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.62</v>
+        <v>-3.31</v>
       </c>
       <c r="D83" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>12</v>
       </c>
       <c r="C84" t="n">
-        <v>4.87</v>
+        <v>5.3</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -1896,7 +1896,7 @@
         <v>13</v>
       </c>
       <c r="C85" t="n">
-        <v>1.32</v>
+        <v>0.57</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -1913,7 +1913,7 @@
         <v>6</v>
       </c>
       <c r="C86" t="n">
-        <v>1.61</v>
+        <v>0.84</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -1930,7 +1930,7 @@
         <v>8</v>
       </c>
       <c r="C87" t="n">
-        <v>-7.04</v>
+        <v>-4.29</v>
       </c>
       <c r="D87" t="n">
         <v>0</v>
@@ -1947,7 +1947,7 @@
         <v>9</v>
       </c>
       <c r="C88" t="n">
-        <v>6.98</v>
+        <v>6.42</v>
       </c>
       <c r="D88" t="n">
         <v>1</v>
@@ -1964,7 +1964,7 @@
         <v>10</v>
       </c>
       <c r="C89" t="n">
-        <v>5.57</v>
+        <v>5.46</v>
       </c>
       <c r="D89" t="n">
         <v>0</v>
@@ -1981,7 +1981,7 @@
         <v>11</v>
       </c>
       <c r="C90" t="n">
-        <v>-7.86</v>
+        <v>-8.72</v>
       </c>
       <c r="D90" t="n">
         <v>0</v>
@@ -1998,7 +1998,7 @@
         <v>12</v>
       </c>
       <c r="C91" t="n">
-        <v>-1.39</v>
+        <v>-1.2</v>
       </c>
       <c r="D91" t="n">
         <v>0</v>
@@ -2015,7 +2015,7 @@
         <v>13</v>
       </c>
       <c r="C92" t="n">
-        <v>2.14</v>
+        <v>1.49</v>
       </c>
       <c r="D92" t="n">
         <v>0</v>
@@ -2032,7 +2032,7 @@
         <v>6</v>
       </c>
       <c r="C93" t="n">
-        <v>2.77</v>
+        <v>1.76</v>
       </c>
       <c r="D93" t="n">
         <v>0</v>
@@ -2049,7 +2049,7 @@
         <v>8</v>
       </c>
       <c r="C94" t="n">
-        <v>-5.31</v>
+        <v>-5.05</v>
       </c>
       <c r="D94" t="n">
         <v>0</v>
@@ -2066,7 +2066,7 @@
         <v>9</v>
       </c>
       <c r="C95" t="n">
-        <v>3.02</v>
+        <v>1.78</v>
       </c>
       <c r="D95" t="n">
         <v>0</v>
@@ -2083,7 +2083,7 @@
         <v>10</v>
       </c>
       <c r="C96" t="n">
-        <v>4.39</v>
+        <v>5.25</v>
       </c>
       <c r="D96" t="n">
         <v>1</v>
@@ -2100,7 +2100,7 @@
         <v>11</v>
       </c>
       <c r="C97" t="n">
-        <v>-11.07</v>
+        <v>-8.4</v>
       </c>
       <c r="D97" t="n">
         <v>0</v>
@@ -2117,7 +2117,7 @@
         <v>12</v>
       </c>
       <c r="C98" t="n">
-        <v>3.63</v>
+        <v>4.03</v>
       </c>
       <c r="D98" t="n">
         <v>0</v>
@@ -2134,7 +2134,7 @@
         <v>13</v>
       </c>
       <c r="C99" t="n">
-        <v>2.57</v>
+        <v>0.63</v>
       </c>
       <c r="D99" t="n">
         <v>0</v>
@@ -2151,7 +2151,7 @@
         <v>6</v>
       </c>
       <c r="C100" t="n">
-        <v>5.72</v>
+        <v>7.1</v>
       </c>
       <c r="D100" t="n">
         <v>1</v>
@@ -2168,7 +2168,7 @@
         <v>8</v>
       </c>
       <c r="C101" t="n">
-        <v>-8.42</v>
+        <v>-5.9</v>
       </c>
       <c r="D101" t="n">
         <v>0</v>
@@ -2185,7 +2185,7 @@
         <v>9</v>
       </c>
       <c r="C102" t="n">
-        <v>-2.71</v>
+        <v>0.4</v>
       </c>
       <c r="D102" t="n">
         <v>0</v>
@@ -2202,7 +2202,7 @@
         <v>10</v>
       </c>
       <c r="C103" t="n">
-        <v>2.22</v>
+        <v>2.31</v>
       </c>
       <c r="D103" t="n">
         <v>0</v>
@@ -2219,7 +2219,7 @@
         <v>11</v>
       </c>
       <c r="C104" t="n">
-        <v>-3.09</v>
+        <v>-6.9</v>
       </c>
       <c r="D104" t="n">
         <v>0</v>
@@ -2236,7 +2236,7 @@
         <v>12</v>
       </c>
       <c r="C105" t="n">
-        <v>2.79</v>
+        <v>-0.04</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
@@ -2253,7 +2253,7 @@
         <v>13</v>
       </c>
       <c r="C106" t="n">
-        <v>3.48</v>
+        <v>3.02</v>
       </c>
       <c r="D106" t="n">
         <v>0</v>
@@ -2270,7 +2270,7 @@
         <v>6</v>
       </c>
       <c r="C107" t="n">
-        <v>-0.48</v>
+        <v>-1.35</v>
       </c>
       <c r="D107" t="n">
         <v>0</v>
@@ -2287,7 +2287,7 @@
         <v>8</v>
       </c>
       <c r="C108" t="n">
-        <v>-0.93</v>
+        <v>5.72</v>
       </c>
       <c r="D108" t="n">
         <v>0</v>
@@ -2304,7 +2304,7 @@
         <v>9</v>
       </c>
       <c r="C109" t="n">
-        <v>6.26</v>
+        <v>5.79</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -2321,7 +2321,7 @@
         <v>10</v>
       </c>
       <c r="C110" t="n">
-        <v>3.13</v>
+        <v>2.27</v>
       </c>
       <c r="D110" t="n">
         <v>0</v>
@@ -2338,7 +2338,7 @@
         <v>11</v>
       </c>
       <c r="C111" t="n">
-        <v>-15.89</v>
+        <v>-18.16</v>
       </c>
       <c r="D111" t="n">
         <v>0</v>
@@ -2355,7 +2355,7 @@
         <v>12</v>
       </c>
       <c r="C112" t="n">
-        <v>5.28</v>
+        <v>4.01</v>
       </c>
       <c r="D112" t="n">
         <v>0</v>
@@ -2372,7 +2372,7 @@
         <v>13</v>
       </c>
       <c r="C113" t="n">
-        <v>2.64</v>
+        <v>1.71</v>
       </c>
       <c r="D113" t="n">
         <v>0</v>
@@ -2389,7 +2389,7 @@
         <v>6</v>
       </c>
       <c r="C114" t="n">
-        <v>-9.56</v>
+        <v>-10.24</v>
       </c>
       <c r="D114" t="n">
         <v>0</v>
@@ -2406,7 +2406,7 @@
         <v>8</v>
       </c>
       <c r="C115" t="n">
-        <v>-1.04</v>
+        <v>-0.65</v>
       </c>
       <c r="D115" t="n">
         <v>0</v>
@@ -2423,7 +2423,7 @@
         <v>9</v>
       </c>
       <c r="C116" t="n">
-        <v>1.76</v>
+        <v>1.77</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
@@ -2440,7 +2440,7 @@
         <v>10</v>
       </c>
       <c r="C117" t="n">
-        <v>5.22</v>
+        <v>5.36</v>
       </c>
       <c r="D117" t="n">
         <v>1</v>
@@ -2457,7 +2457,7 @@
         <v>11</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.9</v>
+        <v>-0.74</v>
       </c>
       <c r="D118" t="n">
         <v>0</v>
@@ -2474,7 +2474,7 @@
         <v>12</v>
       </c>
       <c r="C119" t="n">
-        <v>2.32</v>
+        <v>2.3</v>
       </c>
       <c r="D119" t="n">
         <v>0</v>
@@ -2508,7 +2508,7 @@
         <v>6</v>
       </c>
       <c r="C121" t="n">
-        <v>4.48</v>
+        <v>4.37</v>
       </c>
       <c r="D121" t="n">
         <v>0</v>
@@ -2525,7 +2525,7 @@
         <v>8</v>
       </c>
       <c r="C122" t="n">
-        <v>-13.31</v>
+        <v>-10.18</v>
       </c>
       <c r="D122" t="n">
         <v>0</v>
@@ -2542,7 +2542,7 @@
         <v>9</v>
       </c>
       <c r="C123" t="n">
-        <v>3.53</v>
+        <v>3.6</v>
       </c>
       <c r="D123" t="n">
         <v>0</v>
@@ -2559,7 +2559,7 @@
         <v>10</v>
       </c>
       <c r="C124" t="n">
-        <v>2.97</v>
+        <v>1.95</v>
       </c>
       <c r="D124" t="n">
         <v>0</v>
@@ -2576,7 +2576,7 @@
         <v>11</v>
       </c>
       <c r="C125" t="n">
-        <v>-5.79</v>
+        <v>-7.46</v>
       </c>
       <c r="D125" t="n">
         <v>0</v>
@@ -2593,7 +2593,7 @@
         <v>12</v>
       </c>
       <c r="C126" t="n">
-        <v>1.73</v>
+        <v>1.15</v>
       </c>
       <c r="D126" t="n">
         <v>0</v>
@@ -2610,7 +2610,7 @@
         <v>13</v>
       </c>
       <c r="C127" t="n">
-        <v>6.39</v>
+        <v>6.56</v>
       </c>
       <c r="D127" t="n">
         <v>1</v>
@@ -2627,7 +2627,7 @@
         <v>6</v>
       </c>
       <c r="C128" t="n">
-        <v>4.92</v>
+        <v>3.27</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
@@ -2644,7 +2644,7 @@
         <v>8</v>
       </c>
       <c r="C129" t="n">
-        <v>-5.87</v>
+        <v>1.27</v>
       </c>
       <c r="D129" t="n">
         <v>0</v>
@@ -2661,7 +2661,7 @@
         <v>9</v>
       </c>
       <c r="C130" t="n">
-        <v>5.72</v>
+        <v>4.97</v>
       </c>
       <c r="D130" t="n">
         <v>1</v>
@@ -2678,7 +2678,7 @@
         <v>10</v>
       </c>
       <c r="C131" t="n">
-        <v>1.57</v>
+        <v>1.68</v>
       </c>
       <c r="D131" t="n">
         <v>0</v>
@@ -2695,7 +2695,7 @@
         <v>11</v>
       </c>
       <c r="C132" t="n">
-        <v>-6.87</v>
+        <v>-10.89</v>
       </c>
       <c r="D132" t="n">
         <v>0</v>
@@ -2712,7 +2712,7 @@
         <v>12</v>
       </c>
       <c r="C133" t="n">
-        <v>-3.64</v>
+        <v>-5.13</v>
       </c>
       <c r="D133" t="n">
         <v>0</v>
@@ -2729,7 +2729,7 @@
         <v>13</v>
       </c>
       <c r="C134" t="n">
-        <v>4.15</v>
+        <v>4.83</v>
       </c>
       <c r="D134" t="n">
         <v>0</v>
@@ -2746,7 +2746,7 @@
         <v>6</v>
       </c>
       <c r="C135" t="n">
-        <v>3.98</v>
+        <v>3.51</v>
       </c>
       <c r="D135" t="n">
         <v>0</v>
@@ -2763,7 +2763,7 @@
         <v>8</v>
       </c>
       <c r="C136" t="n">
-        <v>-1.98</v>
+        <v>3.41</v>
       </c>
       <c r="D136" t="n">
         <v>0</v>
@@ -2780,7 +2780,7 @@
         <v>9</v>
       </c>
       <c r="C137" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="D137" t="n">
         <v>0</v>
@@ -2797,7 +2797,7 @@
         <v>10</v>
       </c>
       <c r="C138" t="n">
-        <v>2.32</v>
+        <v>1.48</v>
       </c>
       <c r="D138" t="n">
         <v>0</v>
@@ -2814,7 +2814,7 @@
         <v>11</v>
       </c>
       <c r="C139" t="n">
-        <v>-14.62</v>
+        <v>-16.64</v>
       </c>
       <c r="D139" t="n">
         <v>0</v>
@@ -2831,7 +2831,7 @@
         <v>12</v>
       </c>
       <c r="C140" t="n">
-        <v>3.69</v>
+        <v>2.76</v>
       </c>
       <c r="D140" t="n">
         <v>0</v>
@@ -2848,7 +2848,7 @@
         <v>13</v>
       </c>
       <c r="C141" t="n">
-        <v>5.61</v>
+        <v>5.18</v>
       </c>
       <c r="D141" t="n">
         <v>1</v>
@@ -2865,7 +2865,7 @@
         <v>6</v>
       </c>
       <c r="C142" t="n">
-        <v>-6.87</v>
+        <v>-7.8</v>
       </c>
       <c r="D142" t="n">
         <v>0</v>
@@ -2882,7 +2882,7 @@
         <v>8</v>
       </c>
       <c r="C143" t="n">
-        <v>-6.94</v>
+        <v>-3.93</v>
       </c>
       <c r="D143" t="n">
         <v>0</v>
@@ -2899,7 +2899,7 @@
         <v>9</v>
       </c>
       <c r="C144" t="n">
-        <v>4.93</v>
+        <v>4.91</v>
       </c>
       <c r="D144" t="n">
         <v>1</v>
@@ -2916,7 +2916,7 @@
         <v>10</v>
       </c>
       <c r="C145" t="n">
-        <v>4.09</v>
+        <v>3.69</v>
       </c>
       <c r="D145" t="n">
         <v>0</v>
@@ -2933,7 +2933,7 @@
         <v>11</v>
       </c>
       <c r="C146" t="n">
-        <v>-4.11</v>
+        <v>-5.06</v>
       </c>
       <c r="D146" t="n">
         <v>0</v>
@@ -2950,7 +2950,7 @@
         <v>12</v>
       </c>
       <c r="C147" t="n">
-        <v>4.91</v>
+        <v>4.36</v>
       </c>
       <c r="D147" t="n">
         <v>0</v>
@@ -2967,7 +2967,7 @@
         <v>13</v>
       </c>
       <c r="C148" t="n">
-        <v>3.99</v>
+        <v>3.83</v>
       </c>
       <c r="D148" t="n">
         <v>0</v>
@@ -2984,7 +2984,7 @@
         <v>6</v>
       </c>
       <c r="C149" t="n">
-        <v>3.55</v>
+        <v>2.9</v>
       </c>
       <c r="D149" t="n">
         <v>0</v>
@@ -3001,7 +3001,7 @@
         <v>8</v>
       </c>
       <c r="C150" t="n">
-        <v>-5.31</v>
+        <v>-5.26</v>
       </c>
       <c r="D150" t="n">
         <v>0</v>
@@ -3018,7 +3018,7 @@
         <v>9</v>
       </c>
       <c r="C151" t="n">
-        <v>-6.22</v>
+        <v>-5.9</v>
       </c>
       <c r="D151" t="n">
         <v>0</v>
@@ -3035,7 +3035,7 @@
         <v>10</v>
       </c>
       <c r="C152" t="n">
-        <v>2.9</v>
+        <v>4.78</v>
       </c>
       <c r="D152" t="n">
         <v>0</v>
@@ -3052,7 +3052,7 @@
         <v>11</v>
       </c>
       <c r="C153" t="n">
-        <v>-3.15</v>
+        <v>-5.41</v>
       </c>
       <c r="D153" t="n">
         <v>0</v>
@@ -3069,7 +3069,7 @@
         <v>12</v>
       </c>
       <c r="C154" t="n">
-        <v>7.93</v>
+        <v>7.95</v>
       </c>
       <c r="D154" t="n">
         <v>1</v>
@@ -3086,7 +3086,7 @@
         <v>13</v>
       </c>
       <c r="C155" t="n">
-        <v>0.3</v>
+        <v>0.95</v>
       </c>
       <c r="D155" t="n">
         <v>0</v>
@@ -3103,7 +3103,7 @@
         <v>6</v>
       </c>
       <c r="C156" t="n">
-        <v>4.54</v>
+        <v>4.1</v>
       </c>
       <c r="D156" t="n">
         <v>0</v>
@@ -3120,7 +3120,7 @@
         <v>8</v>
       </c>
       <c r="C157" t="n">
-        <v>-6.95</v>
+        <v>6.49</v>
       </c>
       <c r="D157" t="n">
         <v>0</v>
@@ -3137,7 +3137,7 @@
         <v>9</v>
       </c>
       <c r="C158" t="n">
-        <v>8.2</v>
+        <v>8.43</v>
       </c>
       <c r="D158" t="n">
         <v>1</v>
@@ -3154,7 +3154,7 @@
         <v>10</v>
       </c>
       <c r="C159" t="n">
-        <v>1.92</v>
+        <v>-0.59</v>
       </c>
       <c r="D159" t="n">
         <v>0</v>
@@ -3171,7 +3171,7 @@
         <v>11</v>
       </c>
       <c r="C160" t="n">
-        <v>-11.11</v>
+        <v>-16.45</v>
       </c>
       <c r="D160" t="n">
         <v>0</v>
@@ -3188,7 +3188,7 @@
         <v>12</v>
       </c>
       <c r="C161" t="n">
-        <v>0.01</v>
+        <v>-4.05</v>
       </c>
       <c r="D161" t="n">
         <v>0</v>
@@ -3205,7 +3205,7 @@
         <v>13</v>
       </c>
       <c r="C162" t="n">
-        <v>3.38</v>
+        <v>2.06</v>
       </c>
       <c r="D162" t="n">
         <v>0</v>
@@ -3222,7 +3222,7 @@
         <v>6</v>
       </c>
       <c r="C163" t="n">
-        <v>3.18</v>
+        <v>3.03</v>
       </c>
       <c r="D163" t="n">
         <v>0</v>
@@ -3239,7 +3239,7 @@
         <v>8</v>
       </c>
       <c r="C164" t="n">
-        <v>-2.46</v>
+        <v>2.76</v>
       </c>
       <c r="D164" t="n">
         <v>0</v>
@@ -3256,7 +3256,7 @@
         <v>9</v>
       </c>
       <c r="C165" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="D165" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>10</v>
       </c>
       <c r="C166" t="n">
-        <v>2.31</v>
+        <v>2.09</v>
       </c>
       <c r="D166" t="n">
         <v>0</v>
@@ -3290,7 +3290,7 @@
         <v>11</v>
       </c>
       <c r="C167" t="n">
-        <v>-9.24</v>
+        <v>-11.73</v>
       </c>
       <c r="D167" t="n">
         <v>0</v>
@@ -3307,7 +3307,7 @@
         <v>12</v>
       </c>
       <c r="C168" t="n">
-        <v>-0.21</v>
+        <v>-0.91</v>
       </c>
       <c r="D168" t="n">
         <v>0</v>
@@ -3324,7 +3324,7 @@
         <v>13</v>
       </c>
       <c r="C169" t="n">
-        <v>6.29</v>
+        <v>4.69</v>
       </c>
       <c r="D169" t="n">
         <v>1</v>

</xml_diff>